<commit_message>
Add interactive SEPE dashboard charts
</commit_message>
<xml_diff>
--- a/data/figure_workbooks/tasa_cobertura_ccaa_ultimo_periodo.xlsx
+++ b/data/figure_workbooks/tasa_cobertura_ccaa_ultimo_periodo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -421,6 +421,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -456,6 +457,11 @@
           <t>Tasa de cobertura</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="D6" t="inlineStr">
@@ -466,6 +472,9 @@
       <c r="E6" t="n">
         <v>55.40388890087835</v>
       </c>
+      <c r="F6" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="7">
       <c r="D7" t="inlineStr">
@@ -476,6 +485,9 @@
       <c r="E7" t="n">
         <v>66.6231717386176</v>
       </c>
+      <c r="F7" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="8">
       <c r="D8" t="inlineStr">
@@ -486,6 +498,9 @@
       <c r="E8" t="n">
         <v>71.49708635534712</v>
       </c>
+      <c r="F8" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="9">
       <c r="D9" t="inlineStr">
@@ -496,6 +511,9 @@
       <c r="E9" t="n">
         <v>71.58105258581335</v>
       </c>
+      <c r="F9" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="10">
       <c r="D10" t="inlineStr">
@@ -506,6 +524,9 @@
       <c r="E10" t="n">
         <v>74.50876261285183</v>
       </c>
+      <c r="F10" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="11">
       <c r="D11" t="inlineStr">
@@ -516,6 +537,9 @@
       <c r="E11" t="n">
         <v>76.01199626816343</v>
       </c>
+      <c r="F11" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="12">
       <c r="D12" t="inlineStr">
@@ -526,6 +550,9 @@
       <c r="E12" t="n">
         <v>79.17025763271293</v>
       </c>
+      <c r="F12" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="13">
       <c r="D13" t="inlineStr">
@@ -536,6 +563,9 @@
       <c r="E13" t="n">
         <v>79.56267632078105</v>
       </c>
+      <c r="F13" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="14">
       <c r="D14" t="inlineStr">
@@ -546,6 +576,9 @@
       <c r="E14" t="n">
         <v>79.76820303696947</v>
       </c>
+      <c r="F14" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="15">
       <c r="D15" t="inlineStr">
@@ -556,6 +589,9 @@
       <c r="E15" t="n">
         <v>80.59142770775189</v>
       </c>
+      <c r="F15" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="16">
       <c r="D16" t="inlineStr">
@@ -566,6 +602,9 @@
       <c r="E16" t="n">
         <v>81.27211221623007</v>
       </c>
+      <c r="F16" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="17">
       <c r="D17" t="inlineStr">
@@ -576,6 +615,9 @@
       <c r="E17" t="n">
         <v>90.28841379932899</v>
       </c>
+      <c r="F17" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="18">
       <c r="D18" t="inlineStr">
@@ -586,6 +628,9 @@
       <c r="E18" t="n">
         <v>93.49626429021514</v>
       </c>
+      <c r="F18" t="n">
+        <v>78.76943515470354</v>
+      </c>
     </row>
     <row r="19">
       <c r="D19" t="inlineStr">
@@ -595,6 +640,9 @@
       </c>
       <c r="E19" t="n">
         <v>97.89085652331045</v>
+      </c>
+      <c r="F19" t="n">
+        <v>78.76943515470354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>